<commit_message>
Refresh new_grants.xlsx from the latest Simpler.Grants.gov FairBanks eligibility scan.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/opportunities/new_grants.xlsx
+++ b/opportunities/new_grants.xlsx
@@ -678,7 +678,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>CDC-RFA-JG-26-0056 (Centers for Disease Control-GHC). This Notice of Funding Opportunity (NOFO) seeks to build upon activities funded by CDC to support Global Health Security (GHS) through implementation of programs and activities that focus on protecting and improving health globally through partnerships with Ministries of Health a… Est. programme funding USD 75,000,000; award floor Not listed; ceiling Not listed; ~8 award(s). Entity types include: Unrestricted (i.e., open to any type of entity above), subject to any clarification in text field entitled "Additional Information on Eligibility", Small businesses, For profit organizations other than small businesses. FairBanks / FCHIP theme fit: surveillance…</t>
+          <t>CDC-RFA-JG-26-0056 (Centers for Disease Control-GHC). This Notice of Funding Opportunity (NOFO) seeks to build upon activities funded by CDC to support Global Health Security (GHS) through implementation of programs and activities that focus on protecting and improving health globally through partnerships with Ministries of Health a… Est. programme funding USD 75,000,000; award floor Not listed; ceiling Not listed; ~8 award(s). Entity types include: For profit organizations other than small businesses, Unrestricted (i.e., open to any type of entity above), subject to any clarification in text field entitled "Additional Information on Eligibility", Small businesses. FairBanks / FCHIP theme fit: surveillance…</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -735,7 +735,7 @@
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>Unrestricted (i.e., open to any type of entity above), subject to any clarification in text field entitled "Additional Information on Eligibility"; Small businesses; For profit organizations other than small businesses</t>
+          <t>For profit organizations other than small businesses; Unrestricted (i.e., open to any type of entity above), subject to any clarification in text field entitled "Additional Information on Eligibility"; Small businesses</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
@@ -757,7 +757,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>CDC-RFA-JG-26-0054 (Centers for Disease Control-GHC). The purpose of this NOFO is to continue strengthening Uganda"s capacities for rapid detection and effective and efficient response to health threats. The focus of this NOFO is based on gaps outlined by the 2023 Joint External Evaluation of Uganda"s Global Health Security capaciti… Est. programme funding USD 5,000,000; award floor Not listed; ceiling Not listed; ~3 award(s). Entity types include: For profit organizations other than small businesses, Unrestricted (i.e., open to any type of entity above), subject to any clarification in text field entitled "Additional Information on Eligibility", Small businesses. FairBanks / FCHIP…</t>
+          <t>CDC-RFA-JG-26-0054 (Centers for Disease Control-GHC). The purpose of this NOFO is to continue strengthening Uganda"s capacities for rapid detection and effective and efficient response to health threats. The focus of this NOFO is based on gaps outlined by the 2023 Joint External Evaluation of Uganda"s Global Health Security capaciti… Est. programme funding USD 5,000,000; award floor Not listed; ceiling Not listed; ~3 award(s). Entity types include: Small businesses, For profit organizations other than small businesses, Unrestricted (i.e., open to any type of entity above), subject to any clarification in text field entitled "Additional Information on Eligibility". FairBanks / FCHIP…</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -814,7 +814,7 @@
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>For profit organizations other than small businesses; Unrestricted (i.e., open to any type of entity above), subject to any clarification in text field entitled "Additional Information on Eligibility"; Small businesses</t>
+          <t>Small businesses; For profit organizations other than small businesses; Unrestricted (i.e., open to any type of entity above), subject to any clarification in text field entitled "Additional Information on Eligibility"</t>
         </is>
       </c>
       <c r="Q4" s="2" t="inlineStr">
@@ -836,7 +836,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>CDC-RFA-CK-26-0230 (Centers for Disease Control - NCEZID). This Notice of Funding Opportunity (NOFO) aims to support activities that build and strengthen sustainable fungal disease detection, diagnosis, surveillance, and response systems. Activities may address interconnected areas such as system and workforce development, laboratory and… Est. programme funding USD 15,000,000; award floor Not listed; ceiling Not listed; ~10 award(s). Entity types include: Small businesses, For profit organizations other than small businesses. FairBanks / FCHIP theme fit: surveillance / GHS, HIV / infectious, health systems. Ugandan private company path — confirm full NOFO eligibility and foreign-entity rules on Simpler.Grants.gov before drafting.</t>
+          <t>CDC-RFA-CK-26-0230 (Centers for Disease Control - NCEZID). This Notice of Funding Opportunity (NOFO) aims to support activities that build and strengthen sustainable fungal disease detection, diagnosis, surveillance, and response systems. Activities may address interconnected areas such as system and workforce development, laboratory and… Est. programme funding USD 15,000,000; award floor Not listed; ceiling Not listed; ~10 award(s). Entity types include: For profit organizations other than small businesses, Small businesses. FairBanks / FCHIP theme fit: surveillance / GHS, HIV / infectious, health systems. Ugandan private company path — confirm full NOFO eligibility and foreign-entity rules on Simpler.Grants.gov before drafting.</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -893,7 +893,7 @@
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>Small businesses; For profit organizations other than small businesses</t>
+          <t>For profit organizations other than small businesses; Small businesses</t>
         </is>
       </c>
       <c r="Q5" s="2" t="inlineStr">
@@ -1100,7 +1100,7 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>2026-08-10 20:51</t>
+          <t>2026-08-10 20:56</t>
         </is>
       </c>
     </row>
@@ -1232,7 +1232,7 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>opportunities/build_new_opportunities.py</t>
+          <t>opportunities/build_new_grants.py</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add submission confirmation PDF and remove outdated project narrative PDF for CDC-RFA-JG-26-0056 application
Introduce a new submission confirmation PDF that outlines the application processing steps and tracking information for Grants.gov. Additionally, delete the outdated project narrative PDF to streamline documentation and ensure compliance with current submission requirements. Update the project narrative PDF to improve formatting and consistency.
</commit_message>
<xml_diff>
--- a/opportunities/new_grants.xlsx
+++ b/opportunities/new_grants.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\coding\apps\flutter\fairbanks\opportunities\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A80842F-2DD3-4112-973D-6F4E131634EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC4DD08D-7A25-41C0-A8A7-E7AAC303A90A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -858,7 +858,7 @@
       <c r="A2" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="8" t="s">
         <v>18</v>
       </c>
       <c r="C2" s="2" t="s">
@@ -1152,6 +1152,7 @@
   <autoFilter ref="A1:Q7" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <hyperlinks>
     <hyperlink ref="B3" r:id="rId1" xr:uid="{D8E25EBA-8ADC-4B76-BC8B-C3F5C629FB5C}"/>
+    <hyperlink ref="B2" r:id="rId2" xr:uid="{7C0861A4-A4E9-4014-94C3-E46F85274CE4}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>